<commit_message>
Use brand name CRE Assets; sync CSV and workbook with creassets.com
</commit_message>
<xml_diff>
--- a/creassets-real-estate-waterfall-model.xlsx
+++ b/creassets-real-estate-waterfall-model.xlsx
@@ -17,7 +17,7 @@
     <t>Real estate waterfall model (annual, IRR hurdles)</t>
   </si>
   <si>
-    <t>Free from CREAssets — https://creassets.com/tools/real-estate-waterfall-model-excel</t>
+    <t>Free from CRE Assets — https://creassets.com/tools/real-estate-waterfall-model-excel</t>
   </si>
   <si>
     <t/>
@@ -68,7 +68,7 @@
     <t>General information, not legal, tax or investment advice. Your operating agreement, counsel and CPA govern your deal.</t>
   </si>
   <si>
-    <t>CREAssets is software only. It is not a broker-dealer, funding portal, investment adviser or fund administrator. Figures are illustrative sample data.</t>
+    <t>CRE Assets is software only. It is not a broker-dealer, funding portal, investment adviser or fund administrator. Figures are illustrative sample data.</t>
   </si>
   <si>
     <t>Real estate waterfall model — annual, IRR hurdles</t>

</xml_diff>